<commit_message>
data: activos_prueba agrega México, Brasil, Chile, Europa, China e índices globales (367 activos total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/activos_prueba.xlsx
+++ b/activos_prueba.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I247"/>
+  <dimension ref="A1:I409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5185,6 +5185,3044 @@
       <c r="H247" s="17" t="inlineStr"/>
       <c r="I247" s="17" t="inlineStr"/>
     </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES MÉXICO — BMV ──</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr"/>
+      <c r="C248" s="2" t="inlineStr"/>
+      <c r="D248" s="2" t="inlineStr"/>
+      <c r="E248" s="2" t="inlineStr"/>
+      <c r="F248" s="2" t="inlineStr"/>
+      <c r="G248" s="2" t="inlineStr"/>
+      <c r="H248" s="2" t="inlineStr"/>
+      <c r="I248" s="2" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="12" t="inlineStr">
+        <is>
+          <t>AMXL.MX</t>
+        </is>
+      </c>
+      <c r="B249" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C249" s="12" t="inlineStr"/>
+      <c r="D249" s="12" t="inlineStr"/>
+      <c r="E249" s="12" t="inlineStr"/>
+      <c r="F249" s="12" t="inlineStr"/>
+      <c r="G249" s="12" t="inlineStr"/>
+      <c r="H249" s="12" t="inlineStr"/>
+      <c r="I249" s="12" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="12" t="inlineStr">
+        <is>
+          <t>WALMEX.MX</t>
+        </is>
+      </c>
+      <c r="B250" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C250" s="12" t="inlineStr"/>
+      <c r="D250" s="12" t="inlineStr"/>
+      <c r="E250" s="12" t="inlineStr"/>
+      <c r="F250" s="12" t="inlineStr"/>
+      <c r="G250" s="12" t="inlineStr"/>
+      <c r="H250" s="12" t="inlineStr"/>
+      <c r="I250" s="12" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="12" t="inlineStr">
+        <is>
+          <t>FEMSA.MX</t>
+        </is>
+      </c>
+      <c r="B251" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C251" s="12" t="inlineStr"/>
+      <c r="D251" s="12" t="inlineStr"/>
+      <c r="E251" s="12" t="inlineStr"/>
+      <c r="F251" s="12" t="inlineStr"/>
+      <c r="G251" s="12" t="inlineStr"/>
+      <c r="H251" s="12" t="inlineStr"/>
+      <c r="I251" s="12" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="12" t="inlineStr">
+        <is>
+          <t>GFNORTEO.MX</t>
+        </is>
+      </c>
+      <c r="B252" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C252" s="12" t="inlineStr"/>
+      <c r="D252" s="12" t="inlineStr"/>
+      <c r="E252" s="12" t="inlineStr"/>
+      <c r="F252" s="12" t="inlineStr"/>
+      <c r="G252" s="12" t="inlineStr"/>
+      <c r="H252" s="12" t="inlineStr"/>
+      <c r="I252" s="12" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="12" t="inlineStr">
+        <is>
+          <t>GMEXICOB.MX</t>
+        </is>
+      </c>
+      <c r="B253" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C253" s="12" t="inlineStr"/>
+      <c r="D253" s="12" t="inlineStr"/>
+      <c r="E253" s="12" t="inlineStr"/>
+      <c r="F253" s="12" t="inlineStr"/>
+      <c r="G253" s="12" t="inlineStr"/>
+      <c r="H253" s="12" t="inlineStr"/>
+      <c r="I253" s="12" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="12" t="inlineStr">
+        <is>
+          <t>CEMEXCPO.MX</t>
+        </is>
+      </c>
+      <c r="B254" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C254" s="12" t="inlineStr"/>
+      <c r="D254" s="12" t="inlineStr"/>
+      <c r="E254" s="12" t="inlineStr"/>
+      <c r="F254" s="12" t="inlineStr"/>
+      <c r="G254" s="12" t="inlineStr"/>
+      <c r="H254" s="12" t="inlineStr"/>
+      <c r="I254" s="12" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="12" t="inlineStr">
+        <is>
+          <t>KOFUBL.MX</t>
+        </is>
+      </c>
+      <c r="B255" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C255" s="12" t="inlineStr"/>
+      <c r="D255" s="12" t="inlineStr"/>
+      <c r="E255" s="12" t="inlineStr"/>
+      <c r="F255" s="12" t="inlineStr"/>
+      <c r="G255" s="12" t="inlineStr"/>
+      <c r="H255" s="12" t="inlineStr"/>
+      <c r="I255" s="12" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="12" t="inlineStr">
+        <is>
+          <t>BIMBOA.MX</t>
+        </is>
+      </c>
+      <c r="B256" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C256" s="12" t="inlineStr"/>
+      <c r="D256" s="12" t="inlineStr"/>
+      <c r="E256" s="12" t="inlineStr"/>
+      <c r="F256" s="12" t="inlineStr"/>
+      <c r="G256" s="12" t="inlineStr"/>
+      <c r="H256" s="12" t="inlineStr"/>
+      <c r="I256" s="12" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="12" t="inlineStr">
+        <is>
+          <t>AC.MX</t>
+        </is>
+      </c>
+      <c r="B257" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C257" s="12" t="inlineStr"/>
+      <c r="D257" s="12" t="inlineStr"/>
+      <c r="E257" s="12" t="inlineStr"/>
+      <c r="F257" s="12" t="inlineStr"/>
+      <c r="G257" s="12" t="inlineStr"/>
+      <c r="H257" s="12" t="inlineStr"/>
+      <c r="I257" s="12" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="12" t="inlineStr">
+        <is>
+          <t>GCARSOA1.MX</t>
+        </is>
+      </c>
+      <c r="B258" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C258" s="12" t="inlineStr"/>
+      <c r="D258" s="12" t="inlineStr"/>
+      <c r="E258" s="12" t="inlineStr"/>
+      <c r="F258" s="12" t="inlineStr"/>
+      <c r="G258" s="12" t="inlineStr"/>
+      <c r="H258" s="12" t="inlineStr"/>
+      <c r="I258" s="12" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="12" t="inlineStr">
+        <is>
+          <t>PINFRA.MX</t>
+        </is>
+      </c>
+      <c r="B259" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C259" s="12" t="inlineStr"/>
+      <c r="D259" s="12" t="inlineStr"/>
+      <c r="E259" s="12" t="inlineStr"/>
+      <c r="F259" s="12" t="inlineStr"/>
+      <c r="G259" s="12" t="inlineStr"/>
+      <c r="H259" s="12" t="inlineStr"/>
+      <c r="I259" s="12" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="12" t="inlineStr">
+        <is>
+          <t>ASURB.MX</t>
+        </is>
+      </c>
+      <c r="B260" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C260" s="12" t="inlineStr"/>
+      <c r="D260" s="12" t="inlineStr"/>
+      <c r="E260" s="12" t="inlineStr"/>
+      <c r="F260" s="12" t="inlineStr"/>
+      <c r="G260" s="12" t="inlineStr"/>
+      <c r="H260" s="12" t="inlineStr"/>
+      <c r="I260" s="12" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="12" t="inlineStr">
+        <is>
+          <t>OMAB.MX</t>
+        </is>
+      </c>
+      <c r="B261" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C261" s="12" t="inlineStr"/>
+      <c r="D261" s="12" t="inlineStr"/>
+      <c r="E261" s="12" t="inlineStr"/>
+      <c r="F261" s="12" t="inlineStr"/>
+      <c r="G261" s="12" t="inlineStr"/>
+      <c r="H261" s="12" t="inlineStr"/>
+      <c r="I261" s="12" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="12" t="inlineStr">
+        <is>
+          <t>GAPB.MX</t>
+        </is>
+      </c>
+      <c r="B262" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C262" s="12" t="inlineStr"/>
+      <c r="D262" s="12" t="inlineStr"/>
+      <c r="E262" s="12" t="inlineStr"/>
+      <c r="F262" s="12" t="inlineStr"/>
+      <c r="G262" s="12" t="inlineStr"/>
+      <c r="H262" s="12" t="inlineStr"/>
+      <c r="I262" s="12" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="12" t="inlineStr">
+        <is>
+          <t>ALSEA.MX</t>
+        </is>
+      </c>
+      <c r="B263" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C263" s="12" t="inlineStr"/>
+      <c r="D263" s="12" t="inlineStr"/>
+      <c r="E263" s="12" t="inlineStr"/>
+      <c r="F263" s="12" t="inlineStr"/>
+      <c r="G263" s="12" t="inlineStr"/>
+      <c r="H263" s="12" t="inlineStr"/>
+      <c r="I263" s="12" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="12" t="inlineStr">
+        <is>
+          <t>LIVEPOLC-1.MX</t>
+        </is>
+      </c>
+      <c r="B264" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C264" s="12" t="inlineStr"/>
+      <c r="D264" s="12" t="inlineStr"/>
+      <c r="E264" s="12" t="inlineStr"/>
+      <c r="F264" s="12" t="inlineStr"/>
+      <c r="G264" s="12" t="inlineStr"/>
+      <c r="H264" s="12" t="inlineStr"/>
+      <c r="I264" s="12" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="12" t="inlineStr">
+        <is>
+          <t>BOLSAA.MX</t>
+        </is>
+      </c>
+      <c r="B265" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C265" s="12" t="inlineStr"/>
+      <c r="D265" s="12" t="inlineStr"/>
+      <c r="E265" s="12" t="inlineStr"/>
+      <c r="F265" s="12" t="inlineStr"/>
+      <c r="G265" s="12" t="inlineStr"/>
+      <c r="H265" s="12" t="inlineStr"/>
+      <c r="I265" s="12" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="12" t="inlineStr">
+        <is>
+          <t>MEGACPO.MX</t>
+        </is>
+      </c>
+      <c r="B266" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C266" s="12" t="inlineStr"/>
+      <c r="D266" s="12" t="inlineStr"/>
+      <c r="E266" s="12" t="inlineStr"/>
+      <c r="F266" s="12" t="inlineStr"/>
+      <c r="G266" s="12" t="inlineStr"/>
+      <c r="H266" s="12" t="inlineStr"/>
+      <c r="I266" s="12" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="12" t="inlineStr">
+        <is>
+          <t>TLEVISACPO.MX</t>
+        </is>
+      </c>
+      <c r="B267" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C267" s="12" t="inlineStr"/>
+      <c r="D267" s="12" t="inlineStr"/>
+      <c r="E267" s="12" t="inlineStr"/>
+      <c r="F267" s="12" t="inlineStr"/>
+      <c r="G267" s="12" t="inlineStr"/>
+      <c r="H267" s="12" t="inlineStr"/>
+      <c r="I267" s="12" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="12" t="inlineStr">
+        <is>
+          <t>AMX</t>
+        </is>
+      </c>
+      <c r="B268" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C268" s="12" t="inlineStr"/>
+      <c r="D268" s="12" t="inlineStr"/>
+      <c r="E268" s="12" t="inlineStr"/>
+      <c r="F268" s="12" t="inlineStr"/>
+      <c r="G268" s="12" t="inlineStr"/>
+      <c r="H268" s="12" t="inlineStr"/>
+      <c r="I268" s="12" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="12" t="inlineStr">
+        <is>
+          <t>FMX</t>
+        </is>
+      </c>
+      <c r="B269" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C269" s="12" t="inlineStr"/>
+      <c r="D269" s="12" t="inlineStr"/>
+      <c r="E269" s="12" t="inlineStr"/>
+      <c r="F269" s="12" t="inlineStr"/>
+      <c r="G269" s="12" t="inlineStr"/>
+      <c r="H269" s="12" t="inlineStr"/>
+      <c r="I269" s="12" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="12" t="inlineStr">
+        <is>
+          <t>CX</t>
+        </is>
+      </c>
+      <c r="B270" s="12" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C270" s="12" t="inlineStr"/>
+      <c r="D270" s="12" t="inlineStr"/>
+      <c r="E270" s="12" t="inlineStr"/>
+      <c r="F270" s="12" t="inlineStr"/>
+      <c r="G270" s="12" t="inlineStr"/>
+      <c r="H270" s="12" t="inlineStr"/>
+      <c r="I270" s="12" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES BRASIL — B3 ──</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr"/>
+      <c r="C271" s="2" t="inlineStr"/>
+      <c r="D271" s="2" t="inlineStr"/>
+      <c r="E271" s="2" t="inlineStr"/>
+      <c r="F271" s="2" t="inlineStr"/>
+      <c r="G271" s="2" t="inlineStr"/>
+      <c r="H271" s="2" t="inlineStr"/>
+      <c r="I271" s="2" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="13" t="inlineStr">
+        <is>
+          <t>PETR4.SA</t>
+        </is>
+      </c>
+      <c r="B272" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C272" s="13" t="inlineStr"/>
+      <c r="D272" s="13" t="inlineStr"/>
+      <c r="E272" s="13" t="inlineStr"/>
+      <c r="F272" s="13" t="inlineStr"/>
+      <c r="G272" s="13" t="inlineStr"/>
+      <c r="H272" s="13" t="inlineStr"/>
+      <c r="I272" s="13" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="13" t="inlineStr">
+        <is>
+          <t>PETR3.SA</t>
+        </is>
+      </c>
+      <c r="B273" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C273" s="13" t="inlineStr"/>
+      <c r="D273" s="13" t="inlineStr"/>
+      <c r="E273" s="13" t="inlineStr"/>
+      <c r="F273" s="13" t="inlineStr"/>
+      <c r="G273" s="13" t="inlineStr"/>
+      <c r="H273" s="13" t="inlineStr"/>
+      <c r="I273" s="13" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="13" t="inlineStr">
+        <is>
+          <t>VALE3.SA</t>
+        </is>
+      </c>
+      <c r="B274" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C274" s="13" t="inlineStr"/>
+      <c r="D274" s="13" t="inlineStr"/>
+      <c r="E274" s="13" t="inlineStr"/>
+      <c r="F274" s="13" t="inlineStr"/>
+      <c r="G274" s="13" t="inlineStr"/>
+      <c r="H274" s="13" t="inlineStr"/>
+      <c r="I274" s="13" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="13" t="inlineStr">
+        <is>
+          <t>ITUB4.SA</t>
+        </is>
+      </c>
+      <c r="B275" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C275" s="13" t="inlineStr"/>
+      <c r="D275" s="13" t="inlineStr"/>
+      <c r="E275" s="13" t="inlineStr"/>
+      <c r="F275" s="13" t="inlineStr"/>
+      <c r="G275" s="13" t="inlineStr"/>
+      <c r="H275" s="13" t="inlineStr"/>
+      <c r="I275" s="13" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="13" t="inlineStr">
+        <is>
+          <t>BBDC4.SA</t>
+        </is>
+      </c>
+      <c r="B276" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C276" s="13" t="inlineStr"/>
+      <c r="D276" s="13" t="inlineStr"/>
+      <c r="E276" s="13" t="inlineStr"/>
+      <c r="F276" s="13" t="inlineStr"/>
+      <c r="G276" s="13" t="inlineStr"/>
+      <c r="H276" s="13" t="inlineStr"/>
+      <c r="I276" s="13" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="13" t="inlineStr">
+        <is>
+          <t>ABEV3.SA</t>
+        </is>
+      </c>
+      <c r="B277" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C277" s="13" t="inlineStr"/>
+      <c r="D277" s="13" t="inlineStr"/>
+      <c r="E277" s="13" t="inlineStr"/>
+      <c r="F277" s="13" t="inlineStr"/>
+      <c r="G277" s="13" t="inlineStr"/>
+      <c r="H277" s="13" t="inlineStr"/>
+      <c r="I277" s="13" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="13" t="inlineStr">
+        <is>
+          <t>BBAS3.SA</t>
+        </is>
+      </c>
+      <c r="B278" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C278" s="13" t="inlineStr"/>
+      <c r="D278" s="13" t="inlineStr"/>
+      <c r="E278" s="13" t="inlineStr"/>
+      <c r="F278" s="13" t="inlineStr"/>
+      <c r="G278" s="13" t="inlineStr"/>
+      <c r="H278" s="13" t="inlineStr"/>
+      <c r="I278" s="13" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="13" t="inlineStr">
+        <is>
+          <t>B3SA3.SA</t>
+        </is>
+      </c>
+      <c r="B279" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C279" s="13" t="inlineStr"/>
+      <c r="D279" s="13" t="inlineStr"/>
+      <c r="E279" s="13" t="inlineStr"/>
+      <c r="F279" s="13" t="inlineStr"/>
+      <c r="G279" s="13" t="inlineStr"/>
+      <c r="H279" s="13" t="inlineStr"/>
+      <c r="I279" s="13" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="13" t="inlineStr">
+        <is>
+          <t>WEGE3.SA</t>
+        </is>
+      </c>
+      <c r="B280" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C280" s="13" t="inlineStr"/>
+      <c r="D280" s="13" t="inlineStr"/>
+      <c r="E280" s="13" t="inlineStr"/>
+      <c r="F280" s="13" t="inlineStr"/>
+      <c r="G280" s="13" t="inlineStr"/>
+      <c r="H280" s="13" t="inlineStr"/>
+      <c r="I280" s="13" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="13" t="inlineStr">
+        <is>
+          <t>RENT3.SA</t>
+        </is>
+      </c>
+      <c r="B281" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C281" s="13" t="inlineStr"/>
+      <c r="D281" s="13" t="inlineStr"/>
+      <c r="E281" s="13" t="inlineStr"/>
+      <c r="F281" s="13" t="inlineStr"/>
+      <c r="G281" s="13" t="inlineStr"/>
+      <c r="H281" s="13" t="inlineStr"/>
+      <c r="I281" s="13" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="13" t="inlineStr">
+        <is>
+          <t>SUZB3.SA</t>
+        </is>
+      </c>
+      <c r="B282" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C282" s="13" t="inlineStr"/>
+      <c r="D282" s="13" t="inlineStr"/>
+      <c r="E282" s="13" t="inlineStr"/>
+      <c r="F282" s="13" t="inlineStr"/>
+      <c r="G282" s="13" t="inlineStr"/>
+      <c r="H282" s="13" t="inlineStr"/>
+      <c r="I282" s="13" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="13" t="inlineStr">
+        <is>
+          <t>JBSS3.SA</t>
+        </is>
+      </c>
+      <c r="B283" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C283" s="13" t="inlineStr"/>
+      <c r="D283" s="13" t="inlineStr"/>
+      <c r="E283" s="13" t="inlineStr"/>
+      <c r="F283" s="13" t="inlineStr"/>
+      <c r="G283" s="13" t="inlineStr"/>
+      <c r="H283" s="13" t="inlineStr"/>
+      <c r="I283" s="13" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="13" t="inlineStr">
+        <is>
+          <t>EMBR3.SA</t>
+        </is>
+      </c>
+      <c r="B284" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C284" s="13" t="inlineStr"/>
+      <c r="D284" s="13" t="inlineStr"/>
+      <c r="E284" s="13" t="inlineStr"/>
+      <c r="F284" s="13" t="inlineStr"/>
+      <c r="G284" s="13" t="inlineStr"/>
+      <c r="H284" s="13" t="inlineStr"/>
+      <c r="I284" s="13" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="13" t="inlineStr">
+        <is>
+          <t>ITSA4.SA</t>
+        </is>
+      </c>
+      <c r="B285" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C285" s="13" t="inlineStr"/>
+      <c r="D285" s="13" t="inlineStr"/>
+      <c r="E285" s="13" t="inlineStr"/>
+      <c r="F285" s="13" t="inlineStr"/>
+      <c r="G285" s="13" t="inlineStr"/>
+      <c r="H285" s="13" t="inlineStr"/>
+      <c r="I285" s="13" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="13" t="inlineStr">
+        <is>
+          <t>PRIO3.SA</t>
+        </is>
+      </c>
+      <c r="B286" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C286" s="13" t="inlineStr"/>
+      <c r="D286" s="13" t="inlineStr"/>
+      <c r="E286" s="13" t="inlineStr"/>
+      <c r="F286" s="13" t="inlineStr"/>
+      <c r="G286" s="13" t="inlineStr"/>
+      <c r="H286" s="13" t="inlineStr"/>
+      <c r="I286" s="13" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="13" t="inlineStr">
+        <is>
+          <t>EGIE3.SA</t>
+        </is>
+      </c>
+      <c r="B287" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C287" s="13" t="inlineStr"/>
+      <c r="D287" s="13" t="inlineStr"/>
+      <c r="E287" s="13" t="inlineStr"/>
+      <c r="F287" s="13" t="inlineStr"/>
+      <c r="G287" s="13" t="inlineStr"/>
+      <c r="H287" s="13" t="inlineStr"/>
+      <c r="I287" s="13" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="13" t="inlineStr">
+        <is>
+          <t>RDOR3.SA</t>
+        </is>
+      </c>
+      <c r="B288" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C288" s="13" t="inlineStr"/>
+      <c r="D288" s="13" t="inlineStr"/>
+      <c r="E288" s="13" t="inlineStr"/>
+      <c r="F288" s="13" t="inlineStr"/>
+      <c r="G288" s="13" t="inlineStr"/>
+      <c r="H288" s="13" t="inlineStr"/>
+      <c r="I288" s="13" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="13" t="inlineStr">
+        <is>
+          <t>CSAN3.SA</t>
+        </is>
+      </c>
+      <c r="B289" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C289" s="13" t="inlineStr"/>
+      <c r="D289" s="13" t="inlineStr"/>
+      <c r="E289" s="13" t="inlineStr"/>
+      <c r="F289" s="13" t="inlineStr"/>
+      <c r="G289" s="13" t="inlineStr"/>
+      <c r="H289" s="13" t="inlineStr"/>
+      <c r="I289" s="13" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="13" t="inlineStr">
+        <is>
+          <t>LREN3.SA</t>
+        </is>
+      </c>
+      <c r="B290" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C290" s="13" t="inlineStr"/>
+      <c r="D290" s="13" t="inlineStr"/>
+      <c r="E290" s="13" t="inlineStr"/>
+      <c r="F290" s="13" t="inlineStr"/>
+      <c r="G290" s="13" t="inlineStr"/>
+      <c r="H290" s="13" t="inlineStr"/>
+      <c r="I290" s="13" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="13" t="inlineStr">
+        <is>
+          <t>HAPV3.SA</t>
+        </is>
+      </c>
+      <c r="B291" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C291" s="13" t="inlineStr"/>
+      <c r="D291" s="13" t="inlineStr"/>
+      <c r="E291" s="13" t="inlineStr"/>
+      <c r="F291" s="13" t="inlineStr"/>
+      <c r="G291" s="13" t="inlineStr"/>
+      <c r="H291" s="13" t="inlineStr"/>
+      <c r="I291" s="13" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="13" t="inlineStr">
+        <is>
+          <t>MGLU3.SA</t>
+        </is>
+      </c>
+      <c r="B292" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C292" s="13" t="inlineStr"/>
+      <c r="D292" s="13" t="inlineStr"/>
+      <c r="E292" s="13" t="inlineStr"/>
+      <c r="F292" s="13" t="inlineStr"/>
+      <c r="G292" s="13" t="inlineStr"/>
+      <c r="H292" s="13" t="inlineStr"/>
+      <c r="I292" s="13" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="13" t="inlineStr">
+        <is>
+          <t>AZUL4.SA</t>
+        </is>
+      </c>
+      <c r="B293" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C293" s="13" t="inlineStr"/>
+      <c r="D293" s="13" t="inlineStr"/>
+      <c r="E293" s="13" t="inlineStr"/>
+      <c r="F293" s="13" t="inlineStr"/>
+      <c r="G293" s="13" t="inlineStr"/>
+      <c r="H293" s="13" t="inlineStr"/>
+      <c r="I293" s="13" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="13" t="inlineStr">
+        <is>
+          <t>GOLL4.SA</t>
+        </is>
+      </c>
+      <c r="B294" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C294" s="13" t="inlineStr"/>
+      <c r="D294" s="13" t="inlineStr"/>
+      <c r="E294" s="13" t="inlineStr"/>
+      <c r="F294" s="13" t="inlineStr"/>
+      <c r="G294" s="13" t="inlineStr"/>
+      <c r="H294" s="13" t="inlineStr"/>
+      <c r="I294" s="13" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="13" t="inlineStr">
+        <is>
+          <t>ENEV3.SA</t>
+        </is>
+      </c>
+      <c r="B295" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C295" s="13" t="inlineStr"/>
+      <c r="D295" s="13" t="inlineStr"/>
+      <c r="E295" s="13" t="inlineStr"/>
+      <c r="F295" s="13" t="inlineStr"/>
+      <c r="G295" s="13" t="inlineStr"/>
+      <c r="H295" s="13" t="inlineStr"/>
+      <c r="I295" s="13" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="13" t="inlineStr">
+        <is>
+          <t>TAEE11.SA</t>
+        </is>
+      </c>
+      <c r="B296" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C296" s="13" t="inlineStr"/>
+      <c r="D296" s="13" t="inlineStr"/>
+      <c r="E296" s="13" t="inlineStr"/>
+      <c r="F296" s="13" t="inlineStr"/>
+      <c r="G296" s="13" t="inlineStr"/>
+      <c r="H296" s="13" t="inlineStr"/>
+      <c r="I296" s="13" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="13" t="inlineStr">
+        <is>
+          <t>PBR</t>
+        </is>
+      </c>
+      <c r="B297" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C297" s="13" t="inlineStr"/>
+      <c r="D297" s="13" t="inlineStr"/>
+      <c r="E297" s="13" t="inlineStr"/>
+      <c r="F297" s="13" t="inlineStr"/>
+      <c r="G297" s="13" t="inlineStr"/>
+      <c r="H297" s="13" t="inlineStr"/>
+      <c r="I297" s="13" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="13" t="inlineStr">
+        <is>
+          <t>VALE</t>
+        </is>
+      </c>
+      <c r="B298" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C298" s="13" t="inlineStr"/>
+      <c r="D298" s="13" t="inlineStr"/>
+      <c r="E298" s="13" t="inlineStr"/>
+      <c r="F298" s="13" t="inlineStr"/>
+      <c r="G298" s="13" t="inlineStr"/>
+      <c r="H298" s="13" t="inlineStr"/>
+      <c r="I298" s="13" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="13" t="inlineStr">
+        <is>
+          <t>ITUB</t>
+        </is>
+      </c>
+      <c r="B299" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C299" s="13" t="inlineStr"/>
+      <c r="D299" s="13" t="inlineStr"/>
+      <c r="E299" s="13" t="inlineStr"/>
+      <c r="F299" s="13" t="inlineStr"/>
+      <c r="G299" s="13" t="inlineStr"/>
+      <c r="H299" s="13" t="inlineStr"/>
+      <c r="I299" s="13" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="13" t="inlineStr">
+        <is>
+          <t>BBD</t>
+        </is>
+      </c>
+      <c r="B300" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C300" s="13" t="inlineStr"/>
+      <c r="D300" s="13" t="inlineStr"/>
+      <c r="E300" s="13" t="inlineStr"/>
+      <c r="F300" s="13" t="inlineStr"/>
+      <c r="G300" s="13" t="inlineStr"/>
+      <c r="H300" s="13" t="inlineStr"/>
+      <c r="I300" s="13" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="13" t="inlineStr">
+        <is>
+          <t>ABEV</t>
+        </is>
+      </c>
+      <c r="B301" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C301" s="13" t="inlineStr"/>
+      <c r="D301" s="13" t="inlineStr"/>
+      <c r="E301" s="13" t="inlineStr"/>
+      <c r="F301" s="13" t="inlineStr"/>
+      <c r="G301" s="13" t="inlineStr"/>
+      <c r="H301" s="13" t="inlineStr"/>
+      <c r="I301" s="13" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="13" t="inlineStr">
+        <is>
+          <t>ERJ</t>
+        </is>
+      </c>
+      <c r="B302" s="13" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C302" s="13" t="inlineStr"/>
+      <c r="D302" s="13" t="inlineStr"/>
+      <c r="E302" s="13" t="inlineStr"/>
+      <c r="F302" s="13" t="inlineStr"/>
+      <c r="G302" s="13" t="inlineStr"/>
+      <c r="H302" s="13" t="inlineStr"/>
+      <c r="I302" s="13" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES CHILE — BCS ──</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr"/>
+      <c r="C303" s="2" t="inlineStr"/>
+      <c r="D303" s="2" t="inlineStr"/>
+      <c r="E303" s="2" t="inlineStr"/>
+      <c r="F303" s="2" t="inlineStr"/>
+      <c r="G303" s="2" t="inlineStr"/>
+      <c r="H303" s="2" t="inlineStr"/>
+      <c r="I303" s="2" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="17" t="inlineStr">
+        <is>
+          <t>SQM-B.SN</t>
+        </is>
+      </c>
+      <c r="B304" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C304" s="17" t="inlineStr"/>
+      <c r="D304" s="17" t="inlineStr"/>
+      <c r="E304" s="17" t="inlineStr"/>
+      <c r="F304" s="17" t="inlineStr"/>
+      <c r="G304" s="17" t="inlineStr"/>
+      <c r="H304" s="17" t="inlineStr"/>
+      <c r="I304" s="17" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="17" t="inlineStr">
+        <is>
+          <t>COPEC.SN</t>
+        </is>
+      </c>
+      <c r="B305" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C305" s="17" t="inlineStr"/>
+      <c r="D305" s="17" t="inlineStr"/>
+      <c r="E305" s="17" t="inlineStr"/>
+      <c r="F305" s="17" t="inlineStr"/>
+      <c r="G305" s="17" t="inlineStr"/>
+      <c r="H305" s="17" t="inlineStr"/>
+      <c r="I305" s="17" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="17" t="inlineStr">
+        <is>
+          <t>FALABELLA.SN</t>
+        </is>
+      </c>
+      <c r="B306" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C306" s="17" t="inlineStr"/>
+      <c r="D306" s="17" t="inlineStr"/>
+      <c r="E306" s="17" t="inlineStr"/>
+      <c r="F306" s="17" t="inlineStr"/>
+      <c r="G306" s="17" t="inlineStr"/>
+      <c r="H306" s="17" t="inlineStr"/>
+      <c r="I306" s="17" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="17" t="inlineStr">
+        <is>
+          <t>CENCOSUD.SN</t>
+        </is>
+      </c>
+      <c r="B307" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C307" s="17" t="inlineStr"/>
+      <c r="D307" s="17" t="inlineStr"/>
+      <c r="E307" s="17" t="inlineStr"/>
+      <c r="F307" s="17" t="inlineStr"/>
+      <c r="G307" s="17" t="inlineStr"/>
+      <c r="H307" s="17" t="inlineStr"/>
+      <c r="I307" s="17" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="17" t="inlineStr">
+        <is>
+          <t>CMPC.SN</t>
+        </is>
+      </c>
+      <c r="B308" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C308" s="17" t="inlineStr"/>
+      <c r="D308" s="17" t="inlineStr"/>
+      <c r="E308" s="17" t="inlineStr"/>
+      <c r="F308" s="17" t="inlineStr"/>
+      <c r="G308" s="17" t="inlineStr"/>
+      <c r="H308" s="17" t="inlineStr"/>
+      <c r="I308" s="17" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="17" t="inlineStr">
+        <is>
+          <t>ENELAM.SN</t>
+        </is>
+      </c>
+      <c r="B309" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C309" s="17" t="inlineStr"/>
+      <c r="D309" s="17" t="inlineStr"/>
+      <c r="E309" s="17" t="inlineStr"/>
+      <c r="F309" s="17" t="inlineStr"/>
+      <c r="G309" s="17" t="inlineStr"/>
+      <c r="H309" s="17" t="inlineStr"/>
+      <c r="I309" s="17" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="17" t="inlineStr">
+        <is>
+          <t>COLBUN.SN</t>
+        </is>
+      </c>
+      <c r="B310" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C310" s="17" t="inlineStr"/>
+      <c r="D310" s="17" t="inlineStr"/>
+      <c r="E310" s="17" t="inlineStr"/>
+      <c r="F310" s="17" t="inlineStr"/>
+      <c r="G310" s="17" t="inlineStr"/>
+      <c r="H310" s="17" t="inlineStr"/>
+      <c r="I310" s="17" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="17" t="inlineStr">
+        <is>
+          <t>CCU.SN</t>
+        </is>
+      </c>
+      <c r="B311" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C311" s="17" t="inlineStr"/>
+      <c r="D311" s="17" t="inlineStr"/>
+      <c r="E311" s="17" t="inlineStr"/>
+      <c r="F311" s="17" t="inlineStr"/>
+      <c r="G311" s="17" t="inlineStr"/>
+      <c r="H311" s="17" t="inlineStr"/>
+      <c r="I311" s="17" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="17" t="inlineStr">
+        <is>
+          <t>CHILE.SN</t>
+        </is>
+      </c>
+      <c r="B312" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C312" s="17" t="inlineStr"/>
+      <c r="D312" s="17" t="inlineStr"/>
+      <c r="E312" s="17" t="inlineStr"/>
+      <c r="F312" s="17" t="inlineStr"/>
+      <c r="G312" s="17" t="inlineStr"/>
+      <c r="H312" s="17" t="inlineStr"/>
+      <c r="I312" s="17" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="17" t="inlineStr">
+        <is>
+          <t>BCI.SN</t>
+        </is>
+      </c>
+      <c r="B313" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C313" s="17" t="inlineStr"/>
+      <c r="D313" s="17" t="inlineStr"/>
+      <c r="E313" s="17" t="inlineStr"/>
+      <c r="F313" s="17" t="inlineStr"/>
+      <c r="G313" s="17" t="inlineStr"/>
+      <c r="H313" s="17" t="inlineStr"/>
+      <c r="I313" s="17" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="17" t="inlineStr">
+        <is>
+          <t>SANTANDER.SN</t>
+        </is>
+      </c>
+      <c r="B314" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C314" s="17" t="inlineStr"/>
+      <c r="D314" s="17" t="inlineStr"/>
+      <c r="E314" s="17" t="inlineStr"/>
+      <c r="F314" s="17" t="inlineStr"/>
+      <c r="G314" s="17" t="inlineStr"/>
+      <c r="H314" s="17" t="inlineStr"/>
+      <c r="I314" s="17" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="17" t="inlineStr">
+        <is>
+          <t>AGUAS-A.SN</t>
+        </is>
+      </c>
+      <c r="B315" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C315" s="17" t="inlineStr"/>
+      <c r="D315" s="17" t="inlineStr"/>
+      <c r="E315" s="17" t="inlineStr"/>
+      <c r="F315" s="17" t="inlineStr"/>
+      <c r="G315" s="17" t="inlineStr"/>
+      <c r="H315" s="17" t="inlineStr"/>
+      <c r="I315" s="17" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="17" t="inlineStr">
+        <is>
+          <t>SQM</t>
+        </is>
+      </c>
+      <c r="B316" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C316" s="17" t="inlineStr"/>
+      <c r="D316" s="17" t="inlineStr"/>
+      <c r="E316" s="17" t="inlineStr"/>
+      <c r="F316" s="17" t="inlineStr"/>
+      <c r="G316" s="17" t="inlineStr"/>
+      <c r="H316" s="17" t="inlineStr"/>
+      <c r="I316" s="17" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES EUROPA — ALEMANIA ──</t>
+        </is>
+      </c>
+      <c r="B317" s="2" t="inlineStr"/>
+      <c r="C317" s="2" t="inlineStr"/>
+      <c r="D317" s="2" t="inlineStr"/>
+      <c r="E317" s="2" t="inlineStr"/>
+      <c r="F317" s="2" t="inlineStr"/>
+      <c r="G317" s="2" t="inlineStr"/>
+      <c r="H317" s="2" t="inlineStr"/>
+      <c r="I317" s="2" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>SAP.DE</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="inlineStr"/>
+      <c r="D318" s="3" t="inlineStr"/>
+      <c r="E318" s="3" t="inlineStr"/>
+      <c r="F318" s="3" t="inlineStr"/>
+      <c r="G318" s="3" t="inlineStr"/>
+      <c r="H318" s="3" t="inlineStr"/>
+      <c r="I318" s="3" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="3" t="inlineStr">
+        <is>
+          <t>SIE.DE</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr"/>
+      <c r="D319" s="3" t="inlineStr"/>
+      <c r="E319" s="3" t="inlineStr"/>
+      <c r="F319" s="3" t="inlineStr"/>
+      <c r="G319" s="3" t="inlineStr"/>
+      <c r="H319" s="3" t="inlineStr"/>
+      <c r="I319" s="3" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="3" t="inlineStr">
+        <is>
+          <t>ALV.DE</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C320" s="3" t="inlineStr"/>
+      <c r="D320" s="3" t="inlineStr"/>
+      <c r="E320" s="3" t="inlineStr"/>
+      <c r="F320" s="3" t="inlineStr"/>
+      <c r="G320" s="3" t="inlineStr"/>
+      <c r="H320" s="3" t="inlineStr"/>
+      <c r="I320" s="3" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="3" t="inlineStr">
+        <is>
+          <t>DTE.DE</t>
+        </is>
+      </c>
+      <c r="B321" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C321" s="3" t="inlineStr"/>
+      <c r="D321" s="3" t="inlineStr"/>
+      <c r="E321" s="3" t="inlineStr"/>
+      <c r="F321" s="3" t="inlineStr"/>
+      <c r="G321" s="3" t="inlineStr"/>
+      <c r="H321" s="3" t="inlineStr"/>
+      <c r="I321" s="3" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>BAYN.DE</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="inlineStr"/>
+      <c r="D322" s="3" t="inlineStr"/>
+      <c r="E322" s="3" t="inlineStr"/>
+      <c r="F322" s="3" t="inlineStr"/>
+      <c r="G322" s="3" t="inlineStr"/>
+      <c r="H322" s="3" t="inlineStr"/>
+      <c r="I322" s="3" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="3" t="inlineStr">
+        <is>
+          <t>BMW.DE</t>
+        </is>
+      </c>
+      <c r="B323" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C323" s="3" t="inlineStr"/>
+      <c r="D323" s="3" t="inlineStr"/>
+      <c r="E323" s="3" t="inlineStr"/>
+      <c r="F323" s="3" t="inlineStr"/>
+      <c r="G323" s="3" t="inlineStr"/>
+      <c r="H323" s="3" t="inlineStr"/>
+      <c r="I323" s="3" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="3" t="inlineStr">
+        <is>
+          <t>MBG.DE</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C324" s="3" t="inlineStr"/>
+      <c r="D324" s="3" t="inlineStr"/>
+      <c r="E324" s="3" t="inlineStr"/>
+      <c r="F324" s="3" t="inlineStr"/>
+      <c r="G324" s="3" t="inlineStr"/>
+      <c r="H324" s="3" t="inlineStr"/>
+      <c r="I324" s="3" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="3" t="inlineStr">
+        <is>
+          <t>VOW3.DE</t>
+        </is>
+      </c>
+      <c r="B325" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C325" s="3" t="inlineStr"/>
+      <c r="D325" s="3" t="inlineStr"/>
+      <c r="E325" s="3" t="inlineStr"/>
+      <c r="F325" s="3" t="inlineStr"/>
+      <c r="G325" s="3" t="inlineStr"/>
+      <c r="H325" s="3" t="inlineStr"/>
+      <c r="I325" s="3" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="3" t="inlineStr">
+        <is>
+          <t>BAS.DE</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C326" s="3" t="inlineStr"/>
+      <c r="D326" s="3" t="inlineStr"/>
+      <c r="E326" s="3" t="inlineStr"/>
+      <c r="F326" s="3" t="inlineStr"/>
+      <c r="G326" s="3" t="inlineStr"/>
+      <c r="H326" s="3" t="inlineStr"/>
+      <c r="I326" s="3" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="3" t="inlineStr">
+        <is>
+          <t>DBK.DE</t>
+        </is>
+      </c>
+      <c r="B327" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C327" s="3" t="inlineStr"/>
+      <c r="D327" s="3" t="inlineStr"/>
+      <c r="E327" s="3" t="inlineStr"/>
+      <c r="F327" s="3" t="inlineStr"/>
+      <c r="G327" s="3" t="inlineStr"/>
+      <c r="H327" s="3" t="inlineStr"/>
+      <c r="I327" s="3" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="3" t="inlineStr">
+        <is>
+          <t>ADS.DE</t>
+        </is>
+      </c>
+      <c r="B328" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C328" s="3" t="inlineStr"/>
+      <c r="D328" s="3" t="inlineStr"/>
+      <c r="E328" s="3" t="inlineStr"/>
+      <c r="F328" s="3" t="inlineStr"/>
+      <c r="G328" s="3" t="inlineStr"/>
+      <c r="H328" s="3" t="inlineStr"/>
+      <c r="I328" s="3" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="3" t="inlineStr">
+        <is>
+          <t>RHM.DE</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C329" s="3" t="inlineStr"/>
+      <c r="D329" s="3" t="inlineStr"/>
+      <c r="E329" s="3" t="inlineStr"/>
+      <c r="F329" s="3" t="inlineStr"/>
+      <c r="G329" s="3" t="inlineStr"/>
+      <c r="H329" s="3" t="inlineStr"/>
+      <c r="I329" s="3" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="3" t="inlineStr">
+        <is>
+          <t>HEN3.DE</t>
+        </is>
+      </c>
+      <c r="B330" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C330" s="3" t="inlineStr"/>
+      <c r="D330" s="3" t="inlineStr"/>
+      <c r="E330" s="3" t="inlineStr"/>
+      <c r="F330" s="3" t="inlineStr"/>
+      <c r="G330" s="3" t="inlineStr"/>
+      <c r="H330" s="3" t="inlineStr"/>
+      <c r="I330" s="3" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="3" t="inlineStr">
+        <is>
+          <t>MRK.DE</t>
+        </is>
+      </c>
+      <c r="B331" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C331" s="3" t="inlineStr"/>
+      <c r="D331" s="3" t="inlineStr"/>
+      <c r="E331" s="3" t="inlineStr"/>
+      <c r="F331" s="3" t="inlineStr"/>
+      <c r="G331" s="3" t="inlineStr"/>
+      <c r="H331" s="3" t="inlineStr"/>
+      <c r="I331" s="3" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES EUROPA — FRANCIA ──</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="inlineStr"/>
+      <c r="C332" s="2" t="inlineStr"/>
+      <c r="D332" s="2" t="inlineStr"/>
+      <c r="E332" s="2" t="inlineStr"/>
+      <c r="F332" s="2" t="inlineStr"/>
+      <c r="G332" s="2" t="inlineStr"/>
+      <c r="H332" s="2" t="inlineStr"/>
+      <c r="I332" s="2" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="6" t="inlineStr">
+        <is>
+          <t>MC.PA</t>
+        </is>
+      </c>
+      <c r="B333" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C333" s="6" t="inlineStr"/>
+      <c r="D333" s="6" t="inlineStr"/>
+      <c r="E333" s="6" t="inlineStr"/>
+      <c r="F333" s="6" t="inlineStr"/>
+      <c r="G333" s="6" t="inlineStr"/>
+      <c r="H333" s="6" t="inlineStr"/>
+      <c r="I333" s="6" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="6" t="inlineStr">
+        <is>
+          <t>OR.PA</t>
+        </is>
+      </c>
+      <c r="B334" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C334" s="6" t="inlineStr"/>
+      <c r="D334" s="6" t="inlineStr"/>
+      <c r="E334" s="6" t="inlineStr"/>
+      <c r="F334" s="6" t="inlineStr"/>
+      <c r="G334" s="6" t="inlineStr"/>
+      <c r="H334" s="6" t="inlineStr"/>
+      <c r="I334" s="6" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="6" t="inlineStr">
+        <is>
+          <t>TTE.PA</t>
+        </is>
+      </c>
+      <c r="B335" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C335" s="6" t="inlineStr"/>
+      <c r="D335" s="6" t="inlineStr"/>
+      <c r="E335" s="6" t="inlineStr"/>
+      <c r="F335" s="6" t="inlineStr"/>
+      <c r="G335" s="6" t="inlineStr"/>
+      <c r="H335" s="6" t="inlineStr"/>
+      <c r="I335" s="6" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="6" t="inlineStr">
+        <is>
+          <t>SAN.PA</t>
+        </is>
+      </c>
+      <c r="B336" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C336" s="6" t="inlineStr"/>
+      <c r="D336" s="6" t="inlineStr"/>
+      <c r="E336" s="6" t="inlineStr"/>
+      <c r="F336" s="6" t="inlineStr"/>
+      <c r="G336" s="6" t="inlineStr"/>
+      <c r="H336" s="6" t="inlineStr"/>
+      <c r="I336" s="6" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="6" t="inlineStr">
+        <is>
+          <t>BNP.PA</t>
+        </is>
+      </c>
+      <c r="B337" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C337" s="6" t="inlineStr"/>
+      <c r="D337" s="6" t="inlineStr"/>
+      <c r="E337" s="6" t="inlineStr"/>
+      <c r="F337" s="6" t="inlineStr"/>
+      <c r="G337" s="6" t="inlineStr"/>
+      <c r="H337" s="6" t="inlineStr"/>
+      <c r="I337" s="6" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="6" t="inlineStr">
+        <is>
+          <t>AIR.PA</t>
+        </is>
+      </c>
+      <c r="B338" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C338" s="6" t="inlineStr"/>
+      <c r="D338" s="6" t="inlineStr"/>
+      <c r="E338" s="6" t="inlineStr"/>
+      <c r="F338" s="6" t="inlineStr"/>
+      <c r="G338" s="6" t="inlineStr"/>
+      <c r="H338" s="6" t="inlineStr"/>
+      <c r="I338" s="6" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="6" t="inlineStr">
+        <is>
+          <t>KER.PA</t>
+        </is>
+      </c>
+      <c r="B339" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C339" s="6" t="inlineStr"/>
+      <c r="D339" s="6" t="inlineStr"/>
+      <c r="E339" s="6" t="inlineStr"/>
+      <c r="F339" s="6" t="inlineStr"/>
+      <c r="G339" s="6" t="inlineStr"/>
+      <c r="H339" s="6" t="inlineStr"/>
+      <c r="I339" s="6" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="6" t="inlineStr">
+        <is>
+          <t>CS.PA</t>
+        </is>
+      </c>
+      <c r="B340" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C340" s="6" t="inlineStr"/>
+      <c r="D340" s="6" t="inlineStr"/>
+      <c r="E340" s="6" t="inlineStr"/>
+      <c r="F340" s="6" t="inlineStr"/>
+      <c r="G340" s="6" t="inlineStr"/>
+      <c r="H340" s="6" t="inlineStr"/>
+      <c r="I340" s="6" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="6" t="inlineStr">
+        <is>
+          <t>DG.PA</t>
+        </is>
+      </c>
+      <c r="B341" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C341" s="6" t="inlineStr"/>
+      <c r="D341" s="6" t="inlineStr"/>
+      <c r="E341" s="6" t="inlineStr"/>
+      <c r="F341" s="6" t="inlineStr"/>
+      <c r="G341" s="6" t="inlineStr"/>
+      <c r="H341" s="6" t="inlineStr"/>
+      <c r="I341" s="6" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="6" t="inlineStr">
+        <is>
+          <t>CAP.PA</t>
+        </is>
+      </c>
+      <c r="B342" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C342" s="6" t="inlineStr"/>
+      <c r="D342" s="6" t="inlineStr"/>
+      <c r="E342" s="6" t="inlineStr"/>
+      <c r="F342" s="6" t="inlineStr"/>
+      <c r="G342" s="6" t="inlineStr"/>
+      <c r="H342" s="6" t="inlineStr"/>
+      <c r="I342" s="6" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="6" t="inlineStr">
+        <is>
+          <t>SGO.PA</t>
+        </is>
+      </c>
+      <c r="B343" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C343" s="6" t="inlineStr"/>
+      <c r="D343" s="6" t="inlineStr"/>
+      <c r="E343" s="6" t="inlineStr"/>
+      <c r="F343" s="6" t="inlineStr"/>
+      <c r="G343" s="6" t="inlineStr"/>
+      <c r="H343" s="6" t="inlineStr"/>
+      <c r="I343" s="6" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES EUROPA — REINO UNIDO ──</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="inlineStr"/>
+      <c r="C344" s="2" t="inlineStr"/>
+      <c r="D344" s="2" t="inlineStr"/>
+      <c r="E344" s="2" t="inlineStr"/>
+      <c r="F344" s="2" t="inlineStr"/>
+      <c r="G344" s="2" t="inlineStr"/>
+      <c r="H344" s="2" t="inlineStr"/>
+      <c r="I344" s="2" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="8" t="inlineStr">
+        <is>
+          <t>SHEL.L</t>
+        </is>
+      </c>
+      <c r="B345" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C345" s="8" t="inlineStr"/>
+      <c r="D345" s="8" t="inlineStr"/>
+      <c r="E345" s="8" t="inlineStr"/>
+      <c r="F345" s="8" t="inlineStr"/>
+      <c r="G345" s="8" t="inlineStr"/>
+      <c r="H345" s="8" t="inlineStr"/>
+      <c r="I345" s="8" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="8" t="inlineStr">
+        <is>
+          <t>AZN.L</t>
+        </is>
+      </c>
+      <c r="B346" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C346" s="8" t="inlineStr"/>
+      <c r="D346" s="8" t="inlineStr"/>
+      <c r="E346" s="8" t="inlineStr"/>
+      <c r="F346" s="8" t="inlineStr"/>
+      <c r="G346" s="8" t="inlineStr"/>
+      <c r="H346" s="8" t="inlineStr"/>
+      <c r="I346" s="8" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="8" t="inlineStr">
+        <is>
+          <t>HSBA.L</t>
+        </is>
+      </c>
+      <c r="B347" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C347" s="8" t="inlineStr"/>
+      <c r="D347" s="8" t="inlineStr"/>
+      <c r="E347" s="8" t="inlineStr"/>
+      <c r="F347" s="8" t="inlineStr"/>
+      <c r="G347" s="8" t="inlineStr"/>
+      <c r="H347" s="8" t="inlineStr"/>
+      <c r="I347" s="8" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="8" t="inlineStr">
+        <is>
+          <t>BP.L</t>
+        </is>
+      </c>
+      <c r="B348" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C348" s="8" t="inlineStr"/>
+      <c r="D348" s="8" t="inlineStr"/>
+      <c r="E348" s="8" t="inlineStr"/>
+      <c r="F348" s="8" t="inlineStr"/>
+      <c r="G348" s="8" t="inlineStr"/>
+      <c r="H348" s="8" t="inlineStr"/>
+      <c r="I348" s="8" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="8" t="inlineStr">
+        <is>
+          <t>GSK.L</t>
+        </is>
+      </c>
+      <c r="B349" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C349" s="8" t="inlineStr"/>
+      <c r="D349" s="8" t="inlineStr"/>
+      <c r="E349" s="8" t="inlineStr"/>
+      <c r="F349" s="8" t="inlineStr"/>
+      <c r="G349" s="8" t="inlineStr"/>
+      <c r="H349" s="8" t="inlineStr"/>
+      <c r="I349" s="8" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="8" t="inlineStr">
+        <is>
+          <t>ULVR.L</t>
+        </is>
+      </c>
+      <c r="B350" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C350" s="8" t="inlineStr"/>
+      <c r="D350" s="8" t="inlineStr"/>
+      <c r="E350" s="8" t="inlineStr"/>
+      <c r="F350" s="8" t="inlineStr"/>
+      <c r="G350" s="8" t="inlineStr"/>
+      <c r="H350" s="8" t="inlineStr"/>
+      <c r="I350" s="8" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="8" t="inlineStr">
+        <is>
+          <t>RIO.L</t>
+        </is>
+      </c>
+      <c r="B351" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C351" s="8" t="inlineStr"/>
+      <c r="D351" s="8" t="inlineStr"/>
+      <c r="E351" s="8" t="inlineStr"/>
+      <c r="F351" s="8" t="inlineStr"/>
+      <c r="G351" s="8" t="inlineStr"/>
+      <c r="H351" s="8" t="inlineStr"/>
+      <c r="I351" s="8" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="8" t="inlineStr">
+        <is>
+          <t>AAL.L</t>
+        </is>
+      </c>
+      <c r="B352" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C352" s="8" t="inlineStr"/>
+      <c r="D352" s="8" t="inlineStr"/>
+      <c r="E352" s="8" t="inlineStr"/>
+      <c r="F352" s="8" t="inlineStr"/>
+      <c r="G352" s="8" t="inlineStr"/>
+      <c r="H352" s="8" t="inlineStr"/>
+      <c r="I352" s="8" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="8" t="inlineStr">
+        <is>
+          <t>LLOY.L</t>
+        </is>
+      </c>
+      <c r="B353" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C353" s="8" t="inlineStr"/>
+      <c r="D353" s="8" t="inlineStr"/>
+      <c r="E353" s="8" t="inlineStr"/>
+      <c r="F353" s="8" t="inlineStr"/>
+      <c r="G353" s="8" t="inlineStr"/>
+      <c r="H353" s="8" t="inlineStr"/>
+      <c r="I353" s="8" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="8" t="inlineStr">
+        <is>
+          <t>BARC.L</t>
+        </is>
+      </c>
+      <c r="B354" s="8" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C354" s="8" t="inlineStr"/>
+      <c r="D354" s="8" t="inlineStr"/>
+      <c r="E354" s="8" t="inlineStr"/>
+      <c r="F354" s="8" t="inlineStr"/>
+      <c r="G354" s="8" t="inlineStr"/>
+      <c r="H354" s="8" t="inlineStr"/>
+      <c r="I354" s="8" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES EUROPA — ESPAÑA / PAÍSES BAJOS / SUIZA ──</t>
+        </is>
+      </c>
+      <c r="B355" s="2" t="inlineStr"/>
+      <c r="C355" s="2" t="inlineStr"/>
+      <c r="D355" s="2" t="inlineStr"/>
+      <c r="E355" s="2" t="inlineStr"/>
+      <c r="F355" s="2" t="inlineStr"/>
+      <c r="G355" s="2" t="inlineStr"/>
+      <c r="H355" s="2" t="inlineStr"/>
+      <c r="I355" s="2" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="7" t="inlineStr">
+        <is>
+          <t>SAN.MC</t>
+        </is>
+      </c>
+      <c r="B356" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C356" s="7" t="inlineStr"/>
+      <c r="D356" s="7" t="inlineStr"/>
+      <c r="E356" s="7" t="inlineStr"/>
+      <c r="F356" s="7" t="inlineStr"/>
+      <c r="G356" s="7" t="inlineStr"/>
+      <c r="H356" s="7" t="inlineStr"/>
+      <c r="I356" s="7" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="7" t="inlineStr">
+        <is>
+          <t>ITX.MC</t>
+        </is>
+      </c>
+      <c r="B357" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C357" s="7" t="inlineStr"/>
+      <c r="D357" s="7" t="inlineStr"/>
+      <c r="E357" s="7" t="inlineStr"/>
+      <c r="F357" s="7" t="inlineStr"/>
+      <c r="G357" s="7" t="inlineStr"/>
+      <c r="H357" s="7" t="inlineStr"/>
+      <c r="I357" s="7" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="7" t="inlineStr">
+        <is>
+          <t>BBVA.MC</t>
+        </is>
+      </c>
+      <c r="B358" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C358" s="7" t="inlineStr"/>
+      <c r="D358" s="7" t="inlineStr"/>
+      <c r="E358" s="7" t="inlineStr"/>
+      <c r="F358" s="7" t="inlineStr"/>
+      <c r="G358" s="7" t="inlineStr"/>
+      <c r="H358" s="7" t="inlineStr"/>
+      <c r="I358" s="7" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="7" t="inlineStr">
+        <is>
+          <t>IBE.MC</t>
+        </is>
+      </c>
+      <c r="B359" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C359" s="7" t="inlineStr"/>
+      <c r="D359" s="7" t="inlineStr"/>
+      <c r="E359" s="7" t="inlineStr"/>
+      <c r="F359" s="7" t="inlineStr"/>
+      <c r="G359" s="7" t="inlineStr"/>
+      <c r="H359" s="7" t="inlineStr"/>
+      <c r="I359" s="7" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="7" t="inlineStr">
+        <is>
+          <t>REP.MC</t>
+        </is>
+      </c>
+      <c r="B360" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C360" s="7" t="inlineStr"/>
+      <c r="D360" s="7" t="inlineStr"/>
+      <c r="E360" s="7" t="inlineStr"/>
+      <c r="F360" s="7" t="inlineStr"/>
+      <c r="G360" s="7" t="inlineStr"/>
+      <c r="H360" s="7" t="inlineStr"/>
+      <c r="I360" s="7" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="7" t="inlineStr">
+        <is>
+          <t>ASML.AS</t>
+        </is>
+      </c>
+      <c r="B361" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C361" s="7" t="inlineStr"/>
+      <c r="D361" s="7" t="inlineStr"/>
+      <c r="E361" s="7" t="inlineStr"/>
+      <c r="F361" s="7" t="inlineStr"/>
+      <c r="G361" s="7" t="inlineStr"/>
+      <c r="H361" s="7" t="inlineStr"/>
+      <c r="I361" s="7" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="7" t="inlineStr">
+        <is>
+          <t>HEIA.AS</t>
+        </is>
+      </c>
+      <c r="B362" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C362" s="7" t="inlineStr"/>
+      <c r="D362" s="7" t="inlineStr"/>
+      <c r="E362" s="7" t="inlineStr"/>
+      <c r="F362" s="7" t="inlineStr"/>
+      <c r="G362" s="7" t="inlineStr"/>
+      <c r="H362" s="7" t="inlineStr"/>
+      <c r="I362" s="7" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="7" t="inlineStr">
+        <is>
+          <t>UNA.AS</t>
+        </is>
+      </c>
+      <c r="B363" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C363" s="7" t="inlineStr"/>
+      <c r="D363" s="7" t="inlineStr"/>
+      <c r="E363" s="7" t="inlineStr"/>
+      <c r="F363" s="7" t="inlineStr"/>
+      <c r="G363" s="7" t="inlineStr"/>
+      <c r="H363" s="7" t="inlineStr"/>
+      <c r="I363" s="7" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="7" t="inlineStr">
+        <is>
+          <t>NESN.SW</t>
+        </is>
+      </c>
+      <c r="B364" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C364" s="7" t="inlineStr"/>
+      <c r="D364" s="7" t="inlineStr"/>
+      <c r="E364" s="7" t="inlineStr"/>
+      <c r="F364" s="7" t="inlineStr"/>
+      <c r="G364" s="7" t="inlineStr"/>
+      <c r="H364" s="7" t="inlineStr"/>
+      <c r="I364" s="7" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="7" t="inlineStr">
+        <is>
+          <t>ROG.SW</t>
+        </is>
+      </c>
+      <c r="B365" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C365" s="7" t="inlineStr"/>
+      <c r="D365" s="7" t="inlineStr"/>
+      <c r="E365" s="7" t="inlineStr"/>
+      <c r="F365" s="7" t="inlineStr"/>
+      <c r="G365" s="7" t="inlineStr"/>
+      <c r="H365" s="7" t="inlineStr"/>
+      <c r="I365" s="7" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="7" t="inlineStr">
+        <is>
+          <t>NOVN.SW</t>
+        </is>
+      </c>
+      <c r="B366" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C366" s="7" t="inlineStr"/>
+      <c r="D366" s="7" t="inlineStr"/>
+      <c r="E366" s="7" t="inlineStr"/>
+      <c r="F366" s="7" t="inlineStr"/>
+      <c r="G366" s="7" t="inlineStr"/>
+      <c r="H366" s="7" t="inlineStr"/>
+      <c r="I366" s="7" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="7" t="inlineStr">
+        <is>
+          <t>UBSG.SW</t>
+        </is>
+      </c>
+      <c r="B367" s="7" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C367" s="7" t="inlineStr"/>
+      <c r="D367" s="7" t="inlineStr"/>
+      <c r="E367" s="7" t="inlineStr"/>
+      <c r="F367" s="7" t="inlineStr"/>
+      <c r="G367" s="7" t="inlineStr"/>
+      <c r="H367" s="7" t="inlineStr"/>
+      <c r="I367" s="7" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES CHINA — HONG KONG ──</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="inlineStr"/>
+      <c r="C368" s="2" t="inlineStr"/>
+      <c r="D368" s="2" t="inlineStr"/>
+      <c r="E368" s="2" t="inlineStr"/>
+      <c r="F368" s="2" t="inlineStr"/>
+      <c r="G368" s="2" t="inlineStr"/>
+      <c r="H368" s="2" t="inlineStr"/>
+      <c r="I368" s="2" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="9" t="inlineStr">
+        <is>
+          <t>0700.HK</t>
+        </is>
+      </c>
+      <c r="B369" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C369" s="9" t="inlineStr"/>
+      <c r="D369" s="9" t="inlineStr"/>
+      <c r="E369" s="9" t="inlineStr"/>
+      <c r="F369" s="9" t="inlineStr"/>
+      <c r="G369" s="9" t="inlineStr"/>
+      <c r="H369" s="9" t="inlineStr"/>
+      <c r="I369" s="9" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="9" t="inlineStr">
+        <is>
+          <t>9988.HK</t>
+        </is>
+      </c>
+      <c r="B370" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C370" s="9" t="inlineStr"/>
+      <c r="D370" s="9" t="inlineStr"/>
+      <c r="E370" s="9" t="inlineStr"/>
+      <c r="F370" s="9" t="inlineStr"/>
+      <c r="G370" s="9" t="inlineStr"/>
+      <c r="H370" s="9" t="inlineStr"/>
+      <c r="I370" s="9" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="9" t="inlineStr">
+        <is>
+          <t>3690.HK</t>
+        </is>
+      </c>
+      <c r="B371" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C371" s="9" t="inlineStr"/>
+      <c r="D371" s="9" t="inlineStr"/>
+      <c r="E371" s="9" t="inlineStr"/>
+      <c r="F371" s="9" t="inlineStr"/>
+      <c r="G371" s="9" t="inlineStr"/>
+      <c r="H371" s="9" t="inlineStr"/>
+      <c r="I371" s="9" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="9" t="inlineStr">
+        <is>
+          <t>9618.HK</t>
+        </is>
+      </c>
+      <c r="B372" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C372" s="9" t="inlineStr"/>
+      <c r="D372" s="9" t="inlineStr"/>
+      <c r="E372" s="9" t="inlineStr"/>
+      <c r="F372" s="9" t="inlineStr"/>
+      <c r="G372" s="9" t="inlineStr"/>
+      <c r="H372" s="9" t="inlineStr"/>
+      <c r="I372" s="9" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="9" t="inlineStr">
+        <is>
+          <t>1810.HK</t>
+        </is>
+      </c>
+      <c r="B373" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C373" s="9" t="inlineStr"/>
+      <c r="D373" s="9" t="inlineStr"/>
+      <c r="E373" s="9" t="inlineStr"/>
+      <c r="F373" s="9" t="inlineStr"/>
+      <c r="G373" s="9" t="inlineStr"/>
+      <c r="H373" s="9" t="inlineStr"/>
+      <c r="I373" s="9" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="9" t="inlineStr">
+        <is>
+          <t>0941.HK</t>
+        </is>
+      </c>
+      <c r="B374" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C374" s="9" t="inlineStr"/>
+      <c r="D374" s="9" t="inlineStr"/>
+      <c r="E374" s="9" t="inlineStr"/>
+      <c r="F374" s="9" t="inlineStr"/>
+      <c r="G374" s="9" t="inlineStr"/>
+      <c r="H374" s="9" t="inlineStr"/>
+      <c r="I374" s="9" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="9" t="inlineStr">
+        <is>
+          <t>1398.HK</t>
+        </is>
+      </c>
+      <c r="B375" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C375" s="9" t="inlineStr"/>
+      <c r="D375" s="9" t="inlineStr"/>
+      <c r="E375" s="9" t="inlineStr"/>
+      <c r="F375" s="9" t="inlineStr"/>
+      <c r="G375" s="9" t="inlineStr"/>
+      <c r="H375" s="9" t="inlineStr"/>
+      <c r="I375" s="9" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="9" t="inlineStr">
+        <is>
+          <t>3988.HK</t>
+        </is>
+      </c>
+      <c r="B376" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C376" s="9" t="inlineStr"/>
+      <c r="D376" s="9" t="inlineStr"/>
+      <c r="E376" s="9" t="inlineStr"/>
+      <c r="F376" s="9" t="inlineStr"/>
+      <c r="G376" s="9" t="inlineStr"/>
+      <c r="H376" s="9" t="inlineStr"/>
+      <c r="I376" s="9" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="9" t="inlineStr">
+        <is>
+          <t>2318.HK</t>
+        </is>
+      </c>
+      <c r="B377" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C377" s="9" t="inlineStr"/>
+      <c r="D377" s="9" t="inlineStr"/>
+      <c r="E377" s="9" t="inlineStr"/>
+      <c r="F377" s="9" t="inlineStr"/>
+      <c r="G377" s="9" t="inlineStr"/>
+      <c r="H377" s="9" t="inlineStr"/>
+      <c r="I377" s="9" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="9" t="inlineStr">
+        <is>
+          <t>1211.HK</t>
+        </is>
+      </c>
+      <c r="B378" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C378" s="9" t="inlineStr"/>
+      <c r="D378" s="9" t="inlineStr"/>
+      <c r="E378" s="9" t="inlineStr"/>
+      <c r="F378" s="9" t="inlineStr"/>
+      <c r="G378" s="9" t="inlineStr"/>
+      <c r="H378" s="9" t="inlineStr"/>
+      <c r="I378" s="9" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="9" t="inlineStr">
+        <is>
+          <t>0388.HK</t>
+        </is>
+      </c>
+      <c r="B379" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C379" s="9" t="inlineStr"/>
+      <c r="D379" s="9" t="inlineStr"/>
+      <c r="E379" s="9" t="inlineStr"/>
+      <c r="F379" s="9" t="inlineStr"/>
+      <c r="G379" s="9" t="inlineStr"/>
+      <c r="H379" s="9" t="inlineStr"/>
+      <c r="I379" s="9" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="9" t="inlineStr">
+        <is>
+          <t>0939.HK</t>
+        </is>
+      </c>
+      <c r="B380" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C380" s="9" t="inlineStr"/>
+      <c r="D380" s="9" t="inlineStr"/>
+      <c r="E380" s="9" t="inlineStr"/>
+      <c r="F380" s="9" t="inlineStr"/>
+      <c r="G380" s="9" t="inlineStr"/>
+      <c r="H380" s="9" t="inlineStr"/>
+      <c r="I380" s="9" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="9" t="inlineStr">
+        <is>
+          <t>0175.HK</t>
+        </is>
+      </c>
+      <c r="B381" s="9" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C381" s="9" t="inlineStr"/>
+      <c r="D381" s="9" t="inlineStr"/>
+      <c r="E381" s="9" t="inlineStr"/>
+      <c r="F381" s="9" t="inlineStr"/>
+      <c r="G381" s="9" t="inlineStr"/>
+      <c r="H381" s="9" t="inlineStr"/>
+      <c r="I381" s="9" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>── ACCIONES CHINA — ADRs USA ──</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="inlineStr"/>
+      <c r="C382" s="2" t="inlineStr"/>
+      <c r="D382" s="2" t="inlineStr"/>
+      <c r="E382" s="2" t="inlineStr"/>
+      <c r="F382" s="2" t="inlineStr"/>
+      <c r="G382" s="2" t="inlineStr"/>
+      <c r="H382" s="2" t="inlineStr"/>
+      <c r="I382" s="2" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="10" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="B383" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C383" s="10" t="inlineStr"/>
+      <c r="D383" s="10" t="inlineStr"/>
+      <c r="E383" s="10" t="inlineStr"/>
+      <c r="F383" s="10" t="inlineStr"/>
+      <c r="G383" s="10" t="inlineStr"/>
+      <c r="H383" s="10" t="inlineStr"/>
+      <c r="I383" s="10" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="10" t="inlineStr">
+        <is>
+          <t>PDD</t>
+        </is>
+      </c>
+      <c r="B384" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C384" s="10" t="inlineStr"/>
+      <c r="D384" s="10" t="inlineStr"/>
+      <c r="E384" s="10" t="inlineStr"/>
+      <c r="F384" s="10" t="inlineStr"/>
+      <c r="G384" s="10" t="inlineStr"/>
+      <c r="H384" s="10" t="inlineStr"/>
+      <c r="I384" s="10" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="10" t="inlineStr">
+        <is>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="B385" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C385" s="10" t="inlineStr"/>
+      <c r="D385" s="10" t="inlineStr"/>
+      <c r="E385" s="10" t="inlineStr"/>
+      <c r="F385" s="10" t="inlineStr"/>
+      <c r="G385" s="10" t="inlineStr"/>
+      <c r="H385" s="10" t="inlineStr"/>
+      <c r="I385" s="10" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="10" t="inlineStr">
+        <is>
+          <t>BIDU</t>
+        </is>
+      </c>
+      <c r="B386" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C386" s="10" t="inlineStr"/>
+      <c r="D386" s="10" t="inlineStr"/>
+      <c r="E386" s="10" t="inlineStr"/>
+      <c r="F386" s="10" t="inlineStr"/>
+      <c r="G386" s="10" t="inlineStr"/>
+      <c r="H386" s="10" t="inlineStr"/>
+      <c r="I386" s="10" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="10" t="inlineStr">
+        <is>
+          <t>NIO</t>
+        </is>
+      </c>
+      <c r="B387" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C387" s="10" t="inlineStr"/>
+      <c r="D387" s="10" t="inlineStr"/>
+      <c r="E387" s="10" t="inlineStr"/>
+      <c r="F387" s="10" t="inlineStr"/>
+      <c r="G387" s="10" t="inlineStr"/>
+      <c r="H387" s="10" t="inlineStr"/>
+      <c r="I387" s="10" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="10" t="inlineStr">
+        <is>
+          <t>XPEV</t>
+        </is>
+      </c>
+      <c r="B388" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C388" s="10" t="inlineStr"/>
+      <c r="D388" s="10" t="inlineStr"/>
+      <c r="E388" s="10" t="inlineStr"/>
+      <c r="F388" s="10" t="inlineStr"/>
+      <c r="G388" s="10" t="inlineStr"/>
+      <c r="H388" s="10" t="inlineStr"/>
+      <c r="I388" s="10" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="10" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="B389" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C389" s="10" t="inlineStr"/>
+      <c r="D389" s="10" t="inlineStr"/>
+      <c r="E389" s="10" t="inlineStr"/>
+      <c r="F389" s="10" t="inlineStr"/>
+      <c r="G389" s="10" t="inlineStr"/>
+      <c r="H389" s="10" t="inlineStr"/>
+      <c r="I389" s="10" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="10" t="inlineStr">
+        <is>
+          <t>NTES</t>
+        </is>
+      </c>
+      <c r="B390" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C390" s="10" t="inlineStr"/>
+      <c r="D390" s="10" t="inlineStr"/>
+      <c r="E390" s="10" t="inlineStr"/>
+      <c r="F390" s="10" t="inlineStr"/>
+      <c r="G390" s="10" t="inlineStr"/>
+      <c r="H390" s="10" t="inlineStr"/>
+      <c r="I390" s="10" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="10" t="inlineStr">
+        <is>
+          <t>TCOM</t>
+        </is>
+      </c>
+      <c r="B391" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C391" s="10" t="inlineStr"/>
+      <c r="D391" s="10" t="inlineStr"/>
+      <c r="E391" s="10" t="inlineStr"/>
+      <c r="F391" s="10" t="inlineStr"/>
+      <c r="G391" s="10" t="inlineStr"/>
+      <c r="H391" s="10" t="inlineStr"/>
+      <c r="I391" s="10" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="10" t="inlineStr">
+        <is>
+          <t>YUMC</t>
+        </is>
+      </c>
+      <c r="B392" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C392" s="10" t="inlineStr"/>
+      <c r="D392" s="10" t="inlineStr"/>
+      <c r="E392" s="10" t="inlineStr"/>
+      <c r="F392" s="10" t="inlineStr"/>
+      <c r="G392" s="10" t="inlineStr"/>
+      <c r="H392" s="10" t="inlineStr"/>
+      <c r="I392" s="10" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="10" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="B393" s="10" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C393" s="10" t="inlineStr"/>
+      <c r="D393" s="10" t="inlineStr"/>
+      <c r="E393" s="10" t="inlineStr"/>
+      <c r="F393" s="10" t="inlineStr"/>
+      <c r="G393" s="10" t="inlineStr"/>
+      <c r="H393" s="10" t="inlineStr"/>
+      <c r="I393" s="10" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>── ÍNDICES EUROPA Y ASIA ──</t>
+        </is>
+      </c>
+      <c r="B394" s="2" t="inlineStr"/>
+      <c r="C394" s="2" t="inlineStr"/>
+      <c r="D394" s="2" t="inlineStr"/>
+      <c r="E394" s="2" t="inlineStr"/>
+      <c r="F394" s="2" t="inlineStr"/>
+      <c r="G394" s="2" t="inlineStr"/>
+      <c r="H394" s="2" t="inlineStr"/>
+      <c r="I394" s="2" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="5" t="inlineStr">
+        <is>
+          <t>^GDAXI</t>
+        </is>
+      </c>
+      <c r="B395" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C395" s="5" t="inlineStr"/>
+      <c r="D395" s="5" t="inlineStr"/>
+      <c r="E395" s="5" t="inlineStr"/>
+      <c r="F395" s="5" t="inlineStr"/>
+      <c r="G395" s="5" t="inlineStr"/>
+      <c r="H395" s="5" t="inlineStr"/>
+      <c r="I395" s="5" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="5" t="inlineStr">
+        <is>
+          <t>^FCHI</t>
+        </is>
+      </c>
+      <c r="B396" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C396" s="5" t="inlineStr"/>
+      <c r="D396" s="5" t="inlineStr"/>
+      <c r="E396" s="5" t="inlineStr"/>
+      <c r="F396" s="5" t="inlineStr"/>
+      <c r="G396" s="5" t="inlineStr"/>
+      <c r="H396" s="5" t="inlineStr"/>
+      <c r="I396" s="5" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="5" t="inlineStr">
+        <is>
+          <t>^IBEX</t>
+        </is>
+      </c>
+      <c r="B397" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C397" s="5" t="inlineStr"/>
+      <c r="D397" s="5" t="inlineStr"/>
+      <c r="E397" s="5" t="inlineStr"/>
+      <c r="F397" s="5" t="inlineStr"/>
+      <c r="G397" s="5" t="inlineStr"/>
+      <c r="H397" s="5" t="inlineStr"/>
+      <c r="I397" s="5" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="5" t="inlineStr">
+        <is>
+          <t>^AEX</t>
+        </is>
+      </c>
+      <c r="B398" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C398" s="5" t="inlineStr"/>
+      <c r="D398" s="5" t="inlineStr"/>
+      <c r="E398" s="5" t="inlineStr"/>
+      <c r="F398" s="5" t="inlineStr"/>
+      <c r="G398" s="5" t="inlineStr"/>
+      <c r="H398" s="5" t="inlineStr"/>
+      <c r="I398" s="5" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="5" t="inlineStr">
+        <is>
+          <t>^SMI</t>
+        </is>
+      </c>
+      <c r="B399" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C399" s="5" t="inlineStr"/>
+      <c r="D399" s="5" t="inlineStr"/>
+      <c r="E399" s="5" t="inlineStr"/>
+      <c r="F399" s="5" t="inlineStr"/>
+      <c r="G399" s="5" t="inlineStr"/>
+      <c r="H399" s="5" t="inlineStr"/>
+      <c r="I399" s="5" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="5" t="inlineStr">
+        <is>
+          <t>^MIB</t>
+        </is>
+      </c>
+      <c r="B400" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C400" s="5" t="inlineStr"/>
+      <c r="D400" s="5" t="inlineStr"/>
+      <c r="E400" s="5" t="inlineStr"/>
+      <c r="F400" s="5" t="inlineStr"/>
+      <c r="G400" s="5" t="inlineStr"/>
+      <c r="H400" s="5" t="inlineStr"/>
+      <c r="I400" s="5" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="5" t="inlineStr">
+        <is>
+          <t>^OSEAX</t>
+        </is>
+      </c>
+      <c r="B401" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C401" s="5" t="inlineStr"/>
+      <c r="D401" s="5" t="inlineStr"/>
+      <c r="E401" s="5" t="inlineStr"/>
+      <c r="F401" s="5" t="inlineStr"/>
+      <c r="G401" s="5" t="inlineStr"/>
+      <c r="H401" s="5" t="inlineStr"/>
+      <c r="I401" s="5" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="5" t="inlineStr">
+        <is>
+          <t>000001.SS</t>
+        </is>
+      </c>
+      <c r="B402" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C402" s="5" t="inlineStr"/>
+      <c r="D402" s="5" t="inlineStr"/>
+      <c r="E402" s="5" t="inlineStr"/>
+      <c r="F402" s="5" t="inlineStr"/>
+      <c r="G402" s="5" t="inlineStr"/>
+      <c r="H402" s="5" t="inlineStr"/>
+      <c r="I402" s="5" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="5" t="inlineStr">
+        <is>
+          <t>399001.SZ</t>
+        </is>
+      </c>
+      <c r="B403" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C403" s="5" t="inlineStr"/>
+      <c r="D403" s="5" t="inlineStr"/>
+      <c r="E403" s="5" t="inlineStr"/>
+      <c r="F403" s="5" t="inlineStr"/>
+      <c r="G403" s="5" t="inlineStr"/>
+      <c r="H403" s="5" t="inlineStr"/>
+      <c r="I403" s="5" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="5" t="inlineStr">
+        <is>
+          <t>^AXJO</t>
+        </is>
+      </c>
+      <c r="B404" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C404" s="5" t="inlineStr"/>
+      <c r="D404" s="5" t="inlineStr"/>
+      <c r="E404" s="5" t="inlineStr"/>
+      <c r="F404" s="5" t="inlineStr"/>
+      <c r="G404" s="5" t="inlineStr"/>
+      <c r="H404" s="5" t="inlineStr"/>
+      <c r="I404" s="5" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="5" t="inlineStr">
+        <is>
+          <t>^STI</t>
+        </is>
+      </c>
+      <c r="B405" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C405" s="5" t="inlineStr"/>
+      <c r="D405" s="5" t="inlineStr"/>
+      <c r="E405" s="5" t="inlineStr"/>
+      <c r="F405" s="5" t="inlineStr"/>
+      <c r="G405" s="5" t="inlineStr"/>
+      <c r="H405" s="5" t="inlineStr"/>
+      <c r="I405" s="5" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="5" t="inlineStr">
+        <is>
+          <t>^KS11</t>
+        </is>
+      </c>
+      <c r="B406" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C406" s="5" t="inlineStr"/>
+      <c r="D406" s="5" t="inlineStr"/>
+      <c r="E406" s="5" t="inlineStr"/>
+      <c r="F406" s="5" t="inlineStr"/>
+      <c r="G406" s="5" t="inlineStr"/>
+      <c r="H406" s="5" t="inlineStr"/>
+      <c r="I406" s="5" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="5" t="inlineStr">
+        <is>
+          <t>^TWII</t>
+        </is>
+      </c>
+      <c r="B407" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C407" s="5" t="inlineStr"/>
+      <c r="D407" s="5" t="inlineStr"/>
+      <c r="E407" s="5" t="inlineStr"/>
+      <c r="F407" s="5" t="inlineStr"/>
+      <c r="G407" s="5" t="inlineStr"/>
+      <c r="H407" s="5" t="inlineStr"/>
+      <c r="I407" s="5" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="5" t="inlineStr">
+        <is>
+          <t>^BSESN</t>
+        </is>
+      </c>
+      <c r="B408" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C408" s="5" t="inlineStr"/>
+      <c r="D408" s="5" t="inlineStr"/>
+      <c r="E408" s="5" t="inlineStr"/>
+      <c r="F408" s="5" t="inlineStr"/>
+      <c r="G408" s="5" t="inlineStr"/>
+      <c r="H408" s="5" t="inlineStr"/>
+      <c r="I408" s="5" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="5" t="inlineStr">
+        <is>
+          <t>^NSEI</t>
+        </is>
+      </c>
+      <c r="B409" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C409" s="5" t="inlineStr"/>
+      <c r="D409" s="5" t="inlineStr"/>
+      <c r="E409" s="5" t="inlineStr"/>
+      <c r="F409" s="5" t="inlineStr"/>
+      <c r="G409" s="5" t="inlineStr"/>
+      <c r="H409" s="5" t="inlineStr"/>
+      <c r="I409" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: eliminar YPFD.BA duplicado en activos_prueba.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/activos_prueba.xlsx
+++ b/activos_prueba.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K550"/>
+  <dimension ref="A1:K549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -10303,7 +10303,7 @@
       <c r="I373" s="7" t="n"/>
       <c r="J373" t="inlineStr">
         <is>
-          <t>^SMI</t>
+          <t>^SSMI</t>
         </is>
       </c>
       <c r="K373" t="inlineStr">
@@ -10332,7 +10332,7 @@
       <c r="I374" s="7" t="n"/>
       <c r="J374" t="inlineStr">
         <is>
-          <t>^SMI</t>
+          <t>^SSMI</t>
         </is>
       </c>
       <c r="K374" t="inlineStr">
@@ -10361,7 +10361,7 @@
       <c r="I375" s="7" t="n"/>
       <c r="J375" t="inlineStr">
         <is>
-          <t>^SMI</t>
+          <t>^SSMI</t>
         </is>
       </c>
       <c r="K375" t="inlineStr">
@@ -10390,7 +10390,7 @@
       <c r="I376" s="7" t="n"/>
       <c r="J376" t="inlineStr">
         <is>
-          <t>^SMI</t>
+          <t>^SSMI</t>
         </is>
       </c>
       <c r="K376" t="inlineStr">
@@ -12546,7 +12546,7 @@
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>YPFD.BA</t>
+          <t>AUSO.BA</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
@@ -12568,7 +12568,7 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>AUSO.BA</t>
+          <t>CECO2.BA</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
@@ -12590,7 +12590,7 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>CECO2.BA</t>
+          <t>GARO.BA</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
@@ -12612,7 +12612,7 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>GARO.BA</t>
+          <t>HAVA.BA</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
@@ -12634,7 +12634,7 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>HAVA.BA</t>
+          <t>INVJ.BA</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
@@ -12656,7 +12656,7 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>INVJ.BA</t>
+          <t>REGE.BA</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
@@ -12678,7 +12678,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>REGE.BA</t>
+          <t>CARC.BA</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -12700,36 +12700,36 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>CARC.BA</t>
-        </is>
-      </c>
-      <c r="B485" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J485" t="inlineStr">
-        <is>
-          <t>^MERV</t>
-        </is>
-      </c>
-      <c r="K485" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ADRs BRASIL adicionales ──</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>── ADRs BRASIL adicionales ──</t>
+          <t>GGB</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>GGB</t>
+          <t>SBS</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -12751,7 +12751,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>SBS</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -12773,7 +12773,7 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>XP</t>
+          <t>NU</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
@@ -12795,7 +12795,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>NU</t>
+          <t>STNE</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
@@ -12817,7 +12817,7 @@
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>STNE</t>
+          <t>PAGS</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
@@ -12839,7 +12839,7 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>PAGS</t>
+          <t>VTEX</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
@@ -12861,7 +12861,7 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>VTEX</t>
+          <t>INTR</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
@@ -12883,7 +12883,7 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>AZUL</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
@@ -12905,7 +12905,7 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>AZUL</t>
+          <t>TIMB</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
@@ -12927,7 +12927,7 @@
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>TIMB</t>
+          <t>SID</t>
         </is>
       </c>
       <c r="B496" t="inlineStr">
@@ -12949,7 +12949,7 @@
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>SID</t>
+          <t>UGP</t>
         </is>
       </c>
       <c r="B497" t="inlineStr">
@@ -12971,7 +12971,7 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>UGP</t>
+          <t>CIG</t>
         </is>
       </c>
       <c r="B498" t="inlineStr">
@@ -12993,36 +12993,36 @@
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>CIG</t>
-        </is>
-      </c>
-      <c r="B499" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J499" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="K499" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ADRs COLOMBIA ──</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>── ADRs COLOMBIA ──</t>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>CIB</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
@@ -13044,36 +13044,36 @@
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="B502" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J502" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="K502" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ADRs CHILE adicionales ──</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>── ADRs CHILE adicionales ──</t>
+          <t>BSAC</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>BSAC</t>
+          <t>LTM</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
@@ -13095,36 +13095,36 @@
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>LTM</t>
-        </is>
-      </c>
-      <c r="B505" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J505" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="K505" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ADRs PERU ──</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>── ADRs PERU ──</t>
+          <t>BAP</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>BAP</t>
+          <t>BVN</t>
         </is>
       </c>
       <c r="B507" t="inlineStr">
@@ -13146,65 +13146,65 @@
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>BVN</t>
-        </is>
-      </c>
-      <c r="B508" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J508" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="K508" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ADRs PANAMA / CENTROAMERICA ──</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>── ADRs PANAMA / CENTROAMERICA ──</t>
+          <t>CPA</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>CPA</t>
-        </is>
-      </c>
-      <c r="B510" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J510" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="K510" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ACCIONES COREA — KRX ──</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>── ACCIONES COREA — KRX ──</t>
+          <t>005930.KS</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>^KS11</t>
+        </is>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>005930.KS</t>
+          <t>000660.KS</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
@@ -13226,7 +13226,7 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>000660.KS</t>
+          <t>035420.KS</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
@@ -13248,7 +13248,7 @@
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>035420.KS</t>
+          <t>005380.KS</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
@@ -13270,7 +13270,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>005380.KS</t>
+          <t>051910.KS</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
@@ -13292,7 +13292,7 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>051910.KS</t>
+          <t>035720.KS</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
@@ -13314,7 +13314,7 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>035720.KS</t>
+          <t>207940.KS</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
@@ -13336,36 +13336,36 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>207940.KS</t>
-        </is>
-      </c>
-      <c r="B518" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J518" t="inlineStr">
-        <is>
-          <t>^KS11</t>
-        </is>
-      </c>
-      <c r="K518" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ACCIONES JAPON adicionales ──</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>── ACCIONES JAPON adicionales ──</t>
+          <t>7267.T</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>^N225</t>
+        </is>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>7267.T</t>
+          <t>7751.T</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
@@ -13387,7 +13387,7 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>7751.T</t>
+          <t>6501.T</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
@@ -13409,7 +13409,7 @@
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>6501.T</t>
+          <t>4502.T</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
@@ -13431,7 +13431,7 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>4502.T</t>
+          <t>8035.T</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
@@ -13453,7 +13453,7 @@
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>8035.T</t>
+          <t>9432.T</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
@@ -13475,7 +13475,7 @@
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>9432.T</t>
+          <t>6902.T</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
@@ -13497,36 +13497,31 @@
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>6902.T</t>
-        </is>
-      </c>
-      <c r="B526" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J526" t="inlineStr">
-        <is>
-          <t>^N225</t>
-        </is>
-      </c>
-      <c r="K526" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ETFs ASIA / MEDIO ORIENTE ──</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>── ETFs ASIA / MEDIO ORIENTE ──</t>
+          <t>EWY</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>SPY</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>EWY</t>
+          <t>EWT</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
@@ -13543,7 +13538,7 @@
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>EWT</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
@@ -13560,7 +13555,7 @@
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>EIDO</t>
         </is>
       </c>
       <c r="B530" t="inlineStr">
@@ -13577,7 +13572,7 @@
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>EIDO</t>
+          <t>THD</t>
         </is>
       </c>
       <c r="B531" t="inlineStr">
@@ -13594,7 +13589,7 @@
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>THD</t>
+          <t>KSA</t>
         </is>
       </c>
       <c r="B532" t="inlineStr">
@@ -13611,7 +13606,7 @@
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>KSA</t>
+          <t>GRAB</t>
         </is>
       </c>
       <c r="B533" t="inlineStr">
@@ -13622,13 +13617,18 @@
       <c r="J533" t="inlineStr">
         <is>
           <t>SPY</t>
+        </is>
+      </c>
+      <c r="K533" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>GRAB</t>
+          <t>VNET</t>
         </is>
       </c>
       <c r="B534" t="inlineStr">
@@ -13650,36 +13650,31 @@
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>VNET</t>
-        </is>
-      </c>
-      <c r="B535" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J535" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="K535" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
+          <t>── ETFs TEMATICOS adicionales ──</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>── ETFs TEMATICOS adicionales ──</t>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>SPY</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>XAR</t>
         </is>
       </c>
       <c r="B537" t="inlineStr">
@@ -13696,7 +13691,7 @@
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>XAR</t>
+          <t>ICLN</t>
         </is>
       </c>
       <c r="B538" t="inlineStr">
@@ -13713,7 +13708,7 @@
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>ICLN</t>
+          <t>FSLR</t>
         </is>
       </c>
       <c r="B539" t="inlineStr">
@@ -13724,13 +13719,18 @@
       <c r="J539" t="inlineStr">
         <is>
           <t>SPY</t>
+        </is>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>FSLR</t>
+          <t>ENPH</t>
         </is>
       </c>
       <c r="B540" t="inlineStr">
@@ -13752,7 +13752,7 @@
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>ENPH</t>
+          <t>BNDX</t>
         </is>
       </c>
       <c r="B541" t="inlineStr">
@@ -13763,18 +13763,13 @@
       <c r="J541" t="inlineStr">
         <is>
           <t>SPY</t>
-        </is>
-      </c>
-      <c r="K541" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>BNDX</t>
+          <t>EMB</t>
         </is>
       </c>
       <c r="B542" t="inlineStr">
@@ -13791,7 +13786,7 @@
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>EMB</t>
+          <t>TIP</t>
         </is>
       </c>
       <c r="B543" t="inlineStr">
@@ -13808,7 +13803,7 @@
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>TIP</t>
+          <t>ILF</t>
         </is>
       </c>
       <c r="B544" t="inlineStr">
@@ -13825,7 +13820,7 @@
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>ILF</t>
+          <t>EWP</t>
         </is>
       </c>
       <c r="B545" t="inlineStr">
@@ -13842,7 +13837,7 @@
     <row r="546">
       <c r="A546" t="inlineStr">
         <is>
-          <t>EWP</t>
+          <t>IEMG</t>
         </is>
       </c>
       <c r="B546" t="inlineStr">
@@ -13859,24 +13854,19 @@
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>IEMG</t>
+          <t>^BVSP</t>
         </is>
       </c>
       <c r="B547" t="inlineStr">
         <is>
           <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="J547" t="inlineStr">
-        <is>
-          <t>SPY</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>^BVSP</t>
+          <t>^MXX</t>
         </is>
       </c>
       <c r="B548" t="inlineStr">
@@ -13888,22 +13878,10 @@
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>^MXX</t>
+          <t>^IPSA</t>
         </is>
       </c>
       <c r="B549" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="550">
-      <c r="A550" t="inlineStr">
-        <is>
-          <t>^IPSA</t>
-        </is>
-      </c>
-      <c r="B550" t="inlineStr">
         <is>
           <t>Yahoo Finance</t>
         </is>

</xml_diff>